<commit_message>
New file addition and devlog updates
Continued work on takeoff, hover, and land. Added new file for that, then logged the results in the devlog.
</commit_message>
<xml_diff>
--- a/devlog/RoadmapChecklist.xlsx
+++ b/devlog/RoadmapChecklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardoanselmo/Library/CloudStorage/GoogleDrive-ljanselmo@gmail.com/My Drive/Creative/GitHub/ROS2-Drone-Swarm/devlog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CF75A8-8910-5A4E-91DC-ABCCBAEF09A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561F8488-FD58-6447-B6BD-0C418B1BB28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17160" xr2:uid="{669D467B-3E02-724A-A9F3-17506D17505C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>Commented every line and learned the blocks and what they do. Created some notes on higher level architecture. Still need to figure out specific code and some jargon but will get there.</t>
+  </si>
+  <si>
+    <t>Successfully added the new variable and understood where and how to add it. Also made my own modification with a track of whether it is flying</t>
   </si>
 </sst>
 </file>
@@ -549,6 +552,12 @@
       <c r="C7" t="s">
         <v>9</v>
       </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C8" t="s">

</xml_diff>

<commit_message>
New File + Devlog Update
Created a new test file (takeoff, go to, land) and updated the devlog for this session
</commit_message>
<xml_diff>
--- a/devlog/RoadmapChecklist.xlsx
+++ b/devlog/RoadmapChecklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardoanselmo/Library/CloudStorage/GoogleDrive-ljanselmo@gmail.com/My Drive/Creative/GitHub/ROS2-Drone-Swarm/devlog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561F8488-FD58-6447-B6BD-0C418B1BB28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B337B8-61B8-6D4A-9FC6-97E0AE20A65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17160" xr2:uid="{669D467B-3E02-724A-A9F3-17506D17505C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -574,6 +574,9 @@
       <c r="C10" t="s">
         <v>11</v>
       </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
@@ -589,6 +592,9 @@
       </c>
       <c r="C13" t="s">
         <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>